<commit_message>
phase 1: completed q quit
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vomela-my.sharepoint.com/personal/nguyen_truong_vomela_com/Documents/Desktop/XL to XML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="8_{CE53BFE4-5B2B-424C-B762-D5E09F08BCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D80F6A1-4FBA-4567-BC0A-A71F1ED53B21}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="8_{CE53BFE4-5B2B-424C-B762-D5E09F08BCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B207207-5EC6-419E-8377-6ED7F09140A9}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{73DE167E-CA1B-454F-B46D-856126A641AF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{73DE167E-CA1B-454F-B46D-856126A641AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Template" sheetId="1" r:id="rId1"/>
     <sheet name="Idea" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Current Template'!$A$1:$W$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Current Template'!$A$1:$S$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Idea!$A$1:$Z$50</definedName>
     <definedName name="INVTINFO">#REF!</definedName>
   </definedNames>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2170" uniqueCount="419">
   <si>
     <t>LineType</t>
   </si>
@@ -1295,9 +1295,6 @@
     <t>09</t>
   </si>
   <si>
-    <t>quantity</t>
-  </si>
-  <si>
     <t>job</t>
   </si>
   <si>
@@ -1310,16 +1307,34 @@
     <t>shipVia</t>
   </si>
   <si>
-    <t>count</t>
-  </si>
-  <si>
     <t>trackingNumber</t>
   </si>
   <si>
-    <t>nost</t>
-  </si>
-  <si>
-    <t>name</t>
+    <t>company</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>1Z5636930398492026</t>
+  </si>
+  <si>
+    <t>1111111111 </t>
+  </si>
+  <si>
+    <t>Rod</t>
+  </si>
+  <si>
+    <t>Campbell</t>
+  </si>
+  <si>
+    <t>(480) 226-2757</t>
+  </si>
+  <si>
+    <t>Elitegraphicsinc@Yahoo.com</t>
+  </si>
+  <si>
+    <t>Suite 103</t>
   </si>
 </sst>
 </file>
@@ -1329,7 +1344,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1438,12 +1453,18 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF182026"/>
+      <color rgb="FF37474F"/>
+      <name val="Lucida Sans Unicode"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF106BA3"/>
       <name val="Lucida Sans Unicode"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1486,8 +1507,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1551,11 +1578,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCFD8DC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCFD8DC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCFD8DC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCFD8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1656,15 +1698,16 @@
     <xf numFmtId="49" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2000,237 +2043,4623 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D039AD8E-82AB-E144-B433-E4C02D4187BA}">
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:W103"/>
   <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.25" style="2" customWidth="1"/>
     <col min="2" max="2" width="13.25" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6" style="1" customWidth="1"/>
-    <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.375" style="3" customWidth="1"/>
-    <col min="9" max="10" width="23.625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="46.625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="24.625" style="1" customWidth="1"/>
-    <col min="13" max="14" width="21.625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="12.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.375" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="10.625" style="1"/>
+    <col min="4" max="4" width="20.25" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.375" style="3" customWidth="1"/>
+    <col min="6" max="7" width="23.625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="46.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="24.625" style="1" customWidth="1"/>
+    <col min="10" max="11" width="21.625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.375" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.625" style="1"/>
+    <col min="17" max="17" width="18.375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="8.25" style="1" customWidth="1"/>
+    <col min="19" max="19" width="9.375" style="2" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.375" style="1" customWidth="1"/>
-    <col min="22" max="22" width="8.25" style="1" customWidth="1"/>
-    <col min="23" max="23" width="9.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="10.625" style="1"/>
+    <col min="21" max="16384" width="10.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="E1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="38" t="s">
         <v>410</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="I1" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="38" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q1" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="R1" s="38" t="s">
+        <v>12</v>
+      </c>
+      <c r="S1" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="T1" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="U1" s="39" t="s">
         <v>405</v>
       </c>
-      <c r="F1" s="39" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>412</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="K1" s="9" t="s">
+      <c r="V1" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" s="39" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="13"/>
+      <c r="E2">
+        <v>38.32</v>
+      </c>
+      <c r="F2" s="13"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40" t="s">
         <v>413</v>
       </c>
-      <c r="L1" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="M1" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="P1" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="R1" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="S1" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="U1" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="V1" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="W1" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="X1" s="8" t="s">
-        <v>406</v>
-      </c>
-      <c r="Y1" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z1" s="41" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="14">
-        <v>45973</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="15">
-        <v>1</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="15">
-        <v>1</v>
-      </c>
-      <c r="G2" s="13"/>
-      <c r="H2">
-        <v>38.32</v>
-      </c>
-      <c r="I2" s="16"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="O2" s="18" t="s">
+        <v>418</v>
+      </c>
       <c r="P2" s="13"/>
       <c r="Q2" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="R2" s="18"/>
-      <c r="S2" s="13"/>
+        <v>259</v>
+      </c>
+      <c r="R2" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S2" s="28">
+        <v>94553</v>
+      </c>
       <c r="T2" s="15">
         <v>1</v>
       </c>
-      <c r="U2" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="V2" s="23" t="s">
+      <c r="U2" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V2" s="17">
+        <v>1</v>
+      </c>
+      <c r="W2" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>412</v>
+      </c>
+      <c r="E3">
+        <v>38.32</v>
+      </c>
+      <c r="F3" s="13"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I3" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>414</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>415</v>
+      </c>
+      <c r="L3" s="40" t="s">
+        <v>416</v>
+      </c>
+      <c r="M3" s="42" t="s">
+        <v>417</v>
+      </c>
+      <c r="N3" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="O3" s="21"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="23" t="s">
+        <v>260</v>
+      </c>
+      <c r="R3" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S3" s="28" t="s">
+        <v>261</v>
+      </c>
+      <c r="T3" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U3" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V3" s="17">
+        <v>1</v>
+      </c>
+      <c r="W3" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4">
+        <v>38.32</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="N4" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q4" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="R4" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="T4" s="22">
+        <v>1</v>
+      </c>
+      <c r="U4" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V4" s="17">
+        <v>1</v>
+      </c>
+      <c r="W4" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5">
+        <v>38.32</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q5" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="R5" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="W2" s="28">
-        <v>94553</v>
-      </c>
-      <c r="X2" s="40">
-        <v>99889</v>
-      </c>
-      <c r="Y2" s="1">
-        <v>7</v>
-      </c>
-      <c r="Z2" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="14">
-        <v>45973</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="15">
-        <v>1</v>
-      </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15">
-        <v>1</v>
-      </c>
-      <c r="G3" s="13"/>
-      <c r="H3">
-        <v>38.32</v>
-      </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="23" t="s">
+      <c r="S5" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="T5" s="22">
+        <v>1</v>
+      </c>
+      <c r="U5" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V5" s="17">
+        <v>1</v>
+      </c>
+      <c r="W5" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6">
+        <v>38.32</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I6" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="N6" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q6" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R6" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S6" s="28">
+        <v>73120</v>
+      </c>
+      <c r="T6" s="22">
+        <v>1</v>
+      </c>
+      <c r="U6" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V6" s="17">
+        <v>1</v>
+      </c>
+      <c r="W6" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7">
+        <v>38.32</v>
+      </c>
+      <c r="H7" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="L3" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="R3" s="21"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="22">
-        <v>1</v>
-      </c>
-      <c r="U3" s="23" t="s">
-        <v>260</v>
-      </c>
-      <c r="V3" s="23" t="s">
+      <c r="I7" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="N7" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q7" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R7" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S7" s="28">
+        <v>73129</v>
+      </c>
+      <c r="T7" s="22">
+        <v>1</v>
+      </c>
+      <c r="U7" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V7" s="17">
+        <v>1</v>
+      </c>
+      <c r="W7" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8">
+        <v>38.32</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="N8" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q8" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="R8" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S8" s="28">
+        <v>94589</v>
+      </c>
+      <c r="T8" s="22">
+        <v>1</v>
+      </c>
+      <c r="U8" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V8" s="17">
+        <v>1</v>
+      </c>
+      <c r="W8" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9">
+        <v>38.32</v>
+      </c>
+      <c r="H9" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="I9" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="N9" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q9" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="R9" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="S9" s="29" t="s">
+        <v>269</v>
+      </c>
+      <c r="T9" s="22">
+        <v>1</v>
+      </c>
+      <c r="U9" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V9" s="17">
+        <v>1</v>
+      </c>
+      <c r="W9" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10">
+        <v>38.32</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="N10" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q10" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="R10" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S10" s="28" t="s">
+        <v>270</v>
+      </c>
+      <c r="T10" s="22">
+        <v>1</v>
+      </c>
+      <c r="U10" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V10" s="17">
+        <v>1</v>
+      </c>
+      <c r="W10" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11">
+        <v>38.32</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="N11" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q11" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R11" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S11" s="28">
+        <v>73131</v>
+      </c>
+      <c r="T11" s="22">
+        <v>1</v>
+      </c>
+      <c r="U11" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V11" s="17">
+        <v>1</v>
+      </c>
+      <c r="W11" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12">
+        <v>38.32</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="N12" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q12" s="23" t="s">
+        <v>271</v>
+      </c>
+      <c r="R12" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="W3" s="28" t="s">
-        <v>261</v>
-      </c>
-      <c r="X3" s="40">
-        <v>99889</v>
-      </c>
-      <c r="Y3" s="1">
-        <v>5</v>
-      </c>
-      <c r="Z3" s="1">
-        <v>10</v>
+      <c r="S12" s="28" t="s">
+        <v>272</v>
+      </c>
+      <c r="T12" s="22">
+        <v>1</v>
+      </c>
+      <c r="U12" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V12" s="17">
+        <v>1</v>
+      </c>
+      <c r="W12" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13">
+        <v>38.32</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="N13" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q13" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="R13" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S13" s="28" t="s">
+        <v>275</v>
+      </c>
+      <c r="T13" s="22">
+        <v>1</v>
+      </c>
+      <c r="U13" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V13" s="17">
+        <v>1</v>
+      </c>
+      <c r="W13" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14">
+        <v>38.32</v>
+      </c>
+      <c r="H14" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="I14" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="N14" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q14" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="R14" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="S14" s="30" t="s">
+        <v>277</v>
+      </c>
+      <c r="T14" s="22">
+        <v>1</v>
+      </c>
+      <c r="U14" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V14" s="17">
+        <v>1</v>
+      </c>
+      <c r="W14" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15">
+        <v>38.32</v>
+      </c>
+      <c r="H15" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="N15" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q15" s="23" t="s">
+        <v>278</v>
+      </c>
+      <c r="R15" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S15" s="28" t="s">
+        <v>279</v>
+      </c>
+      <c r="T15" s="22">
+        <v>1</v>
+      </c>
+      <c r="U15" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V15" s="17">
+        <v>1</v>
+      </c>
+      <c r="W15" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16">
+        <v>38.32</v>
+      </c>
+      <c r="H16" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="N16" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q16" s="23" t="s">
+        <v>280</v>
+      </c>
+      <c r="R16" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S16" s="28">
+        <v>20678</v>
+      </c>
+      <c r="T16" s="22">
+        <v>1</v>
+      </c>
+      <c r="U16" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V16" s="17">
+        <v>1</v>
+      </c>
+      <c r="W16" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17">
+        <v>38.32</v>
+      </c>
+      <c r="H17" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="N17" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q17" s="23" t="s">
+        <v>281</v>
+      </c>
+      <c r="R17" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S17" s="28">
+        <v>73012</v>
+      </c>
+      <c r="T17" s="22">
+        <v>1</v>
+      </c>
+      <c r="U17" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V17" s="17">
+        <v>1</v>
+      </c>
+      <c r="W17" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18">
+        <v>38.32</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I18" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="N18" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q18" s="23" t="s">
+        <v>282</v>
+      </c>
+      <c r="R18" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S18" s="28" t="s">
+        <v>283</v>
+      </c>
+      <c r="T18" s="22">
+        <v>1</v>
+      </c>
+      <c r="U18" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V18" s="17">
+        <v>1</v>
+      </c>
+      <c r="W18" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19">
+        <v>38.32</v>
+      </c>
+      <c r="H19" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="N19" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q19" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="R19" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S19" s="28" t="s">
+        <v>285</v>
+      </c>
+      <c r="T19" s="22">
+        <v>1</v>
+      </c>
+      <c r="U19" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V19" s="17">
+        <v>1</v>
+      </c>
+      <c r="W19" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20">
+        <v>38.32</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I20" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="N20" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q20" s="23" t="s">
+        <v>286</v>
+      </c>
+      <c r="R20" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S20" s="28" t="s">
+        <v>287</v>
+      </c>
+      <c r="T20" s="22">
+        <v>1</v>
+      </c>
+      <c r="U20" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V20" s="17">
+        <v>1</v>
+      </c>
+      <c r="W20" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21">
+        <v>38.32</v>
+      </c>
+      <c r="H21" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I21" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="N21" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q21" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="R21" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="S21" s="28" t="s">
+        <v>289</v>
+      </c>
+      <c r="T21" s="22">
+        <v>1</v>
+      </c>
+      <c r="U21" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V21" s="17">
+        <v>1</v>
+      </c>
+      <c r="W21" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22">
+        <v>38.32</v>
+      </c>
+      <c r="H22" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="N22" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q22" s="23" t="s">
+        <v>290</v>
+      </c>
+      <c r="R22" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S22" s="28">
+        <v>73069</v>
+      </c>
+      <c r="T22" s="22">
+        <v>1</v>
+      </c>
+      <c r="U22" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V22" s="17">
+        <v>1</v>
+      </c>
+      <c r="W22" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23">
+        <v>38.32</v>
+      </c>
+      <c r="H23" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="N23" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q23" s="23" t="s">
+        <v>278</v>
+      </c>
+      <c r="R23" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S23" s="28" t="s">
+        <v>291</v>
+      </c>
+      <c r="T23" s="22">
+        <v>1</v>
+      </c>
+      <c r="U23" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V23" s="17">
+        <v>1</v>
+      </c>
+      <c r="W23" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24">
+        <v>38.32</v>
+      </c>
+      <c r="H24" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="I24" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="N24" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q24" s="23" t="s">
+        <v>292</v>
+      </c>
+      <c r="R24" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S24" s="28" t="s">
+        <v>293</v>
+      </c>
+      <c r="T24" s="22">
+        <v>1</v>
+      </c>
+      <c r="U24" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V24" s="17">
+        <v>1</v>
+      </c>
+      <c r="W24" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25">
+        <v>38.32</v>
+      </c>
+      <c r="H25" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="N25" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q25" s="23" t="s">
+        <v>294</v>
+      </c>
+      <c r="R25" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S25" s="28" t="s">
+        <v>295</v>
+      </c>
+      <c r="T25" s="22">
+        <v>1</v>
+      </c>
+      <c r="U25" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V25" s="17">
+        <v>1</v>
+      </c>
+      <c r="W25" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26">
+        <v>38.32</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="N26" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q26" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="R26" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S26" s="28">
+        <v>77318</v>
+      </c>
+      <c r="T26" s="22">
+        <v>1</v>
+      </c>
+      <c r="U26" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V26" s="17">
+        <v>1</v>
+      </c>
+      <c r="W26" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E27">
+        <v>38.32</v>
+      </c>
+      <c r="H27" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I27" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="N27" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="Q27" s="23" t="s">
+        <v>296</v>
+      </c>
+      <c r="R27" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S27" s="28">
+        <v>73064</v>
+      </c>
+      <c r="T27" s="22">
+        <v>1</v>
+      </c>
+      <c r="U27" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V27" s="17">
+        <v>1</v>
+      </c>
+      <c r="W27" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28">
+        <v>38.32</v>
+      </c>
+      <c r="H28" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I28" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="N28" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q28" s="23" t="s">
+        <v>297</v>
+      </c>
+      <c r="R28" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S28" s="28">
+        <v>91355</v>
+      </c>
+      <c r="T28" s="22">
+        <v>1</v>
+      </c>
+      <c r="U28" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V28" s="17">
+        <v>1</v>
+      </c>
+      <c r="W28" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E29">
+        <v>38.32</v>
+      </c>
+      <c r="H29" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="I29" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="N29" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q29" s="23" t="s">
+        <v>298</v>
+      </c>
+      <c r="R29" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S29" s="28">
+        <v>20747</v>
+      </c>
+      <c r="T29" s="22">
+        <v>1</v>
+      </c>
+      <c r="U29" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V29" s="17">
+        <v>1</v>
+      </c>
+      <c r="W29" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30">
+        <v>38.32</v>
+      </c>
+      <c r="H30" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I30" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="N30" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="Q30" s="23" t="s">
+        <v>299</v>
+      </c>
+      <c r="R30" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S30" s="28" t="s">
+        <v>300</v>
+      </c>
+      <c r="T30" s="22">
+        <v>1</v>
+      </c>
+      <c r="U30" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V30" s="17">
+        <v>1</v>
+      </c>
+      <c r="W30" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="H31" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="I31" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="N31" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q31" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="R31" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="S31" s="31" t="s">
+        <v>302</v>
+      </c>
+      <c r="T31" s="22">
+        <v>1</v>
+      </c>
+      <c r="U31" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V31" s="17">
+        <v>1</v>
+      </c>
+      <c r="W31" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32">
+        <v>38.32</v>
+      </c>
+      <c r="H32" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I32" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="N32" s="25" t="s">
+        <v>187</v>
+      </c>
+      <c r="Q32" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="R32" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="S32" s="29" t="s">
+        <v>303</v>
+      </c>
+      <c r="T32" s="22">
+        <v>1</v>
+      </c>
+      <c r="U32" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V32" s="17">
+        <v>1</v>
+      </c>
+      <c r="W32" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A33" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33">
+        <v>38.32</v>
+      </c>
+      <c r="H33" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="I33" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="N33" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q33" s="23" t="s">
+        <v>304</v>
+      </c>
+      <c r="R33" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S33" s="28" t="s">
+        <v>305</v>
+      </c>
+      <c r="T33" s="22">
+        <v>1</v>
+      </c>
+      <c r="U33" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V33" s="17">
+        <v>1</v>
+      </c>
+      <c r="W33" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A34" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34">
+        <v>38.32</v>
+      </c>
+      <c r="H34" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="I34" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="N34" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q34" s="23" t="s">
+        <v>306</v>
+      </c>
+      <c r="R34" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S34" s="28" t="s">
+        <v>307</v>
+      </c>
+      <c r="T34" s="22">
+        <v>1</v>
+      </c>
+      <c r="U34" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V34" s="17">
+        <v>1</v>
+      </c>
+      <c r="W34" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35">
+        <v>38.32</v>
+      </c>
+      <c r="H35" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I35" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="N35" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q35" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="R35" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S35" s="28">
+        <v>94014</v>
+      </c>
+      <c r="T35" s="22">
+        <v>1</v>
+      </c>
+      <c r="U35" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V35" s="17">
+        <v>1</v>
+      </c>
+      <c r="W35" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A36" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36">
+        <v>38.32</v>
+      </c>
+      <c r="H36" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I36" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="N36" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q36" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="R36" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S36" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="T36" s="22">
+        <v>1</v>
+      </c>
+      <c r="U36" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V36" s="17">
+        <v>1</v>
+      </c>
+      <c r="W36" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A37" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37">
+        <v>38.32</v>
+      </c>
+      <c r="H37" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I37" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="N37" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q37" s="23" t="s">
+        <v>311</v>
+      </c>
+      <c r="R37" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S37" s="28">
+        <v>48439</v>
+      </c>
+      <c r="T37" s="22">
+        <v>1</v>
+      </c>
+      <c r="U37" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V37" s="17">
+        <v>1</v>
+      </c>
+      <c r="W37" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A38" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38">
+        <v>38.32</v>
+      </c>
+      <c r="H38" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I38" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="N38" s="25" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q38" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="R38" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S38" s="29" t="s">
+        <v>313</v>
+      </c>
+      <c r="T38" s="22">
+        <v>1</v>
+      </c>
+      <c r="U38" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V38" s="17">
+        <v>1</v>
+      </c>
+      <c r="W38" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A39" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39">
+        <v>38.32</v>
+      </c>
+      <c r="H39" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="I39" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="N39" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q39" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="R39" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="S39" s="32" t="s">
+        <v>315</v>
+      </c>
+      <c r="T39" s="22">
+        <v>1</v>
+      </c>
+      <c r="U39" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V39" s="17">
+        <v>1</v>
+      </c>
+      <c r="W39" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A40" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E40">
+        <v>38.32</v>
+      </c>
+      <c r="H40" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="I40" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="N40" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q40" s="23" t="s">
+        <v>316</v>
+      </c>
+      <c r="R40" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S40" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="T40" s="22">
+        <v>1</v>
+      </c>
+      <c r="U40" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V40" s="17">
+        <v>1</v>
+      </c>
+      <c r="W40" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A41" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E41">
+        <v>38.32</v>
+      </c>
+      <c r="H41" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I41" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="N41" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q41" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="R41" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S41" s="29" t="s">
+        <v>319</v>
+      </c>
+      <c r="T41" s="22">
+        <v>1</v>
+      </c>
+      <c r="U41" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V41" s="17">
+        <v>1</v>
+      </c>
+      <c r="W41" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A42" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E42">
+        <v>38.32</v>
+      </c>
+      <c r="H42" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I42" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="N42" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q42" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R42" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S42" s="28">
+        <v>73107</v>
+      </c>
+      <c r="T42" s="22">
+        <v>1</v>
+      </c>
+      <c r="U42" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V42" s="17">
+        <v>1</v>
+      </c>
+      <c r="W42" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A43" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E43">
+        <v>38.32</v>
+      </c>
+      <c r="H43" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I43" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="N43" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q43" s="23" t="s">
+        <v>281</v>
+      </c>
+      <c r="R43" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S43" s="28">
+        <v>73013</v>
+      </c>
+      <c r="T43" s="22">
+        <v>1</v>
+      </c>
+      <c r="U43" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V43" s="17">
+        <v>1</v>
+      </c>
+      <c r="W43" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A44" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E44">
+        <v>38.32</v>
+      </c>
+      <c r="H44" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I44" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="N44" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q44" s="23" t="s">
+        <v>320</v>
+      </c>
+      <c r="R44" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S44" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="T44" s="22">
+        <v>1</v>
+      </c>
+      <c r="U44" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V44" s="17">
+        <v>1</v>
+      </c>
+      <c r="W44" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A45" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E45">
+        <v>38.32</v>
+      </c>
+      <c r="H45" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I45" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="N45" s="23" t="s">
+        <v>200</v>
+      </c>
+      <c r="Q45" s="23" t="s">
+        <v>322</v>
+      </c>
+      <c r="R45" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S45" s="28">
+        <v>91606</v>
+      </c>
+      <c r="T45" s="22">
+        <v>1</v>
+      </c>
+      <c r="U45" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V45" s="17">
+        <v>1</v>
+      </c>
+      <c r="W45" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A46" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46">
+        <v>38.32</v>
+      </c>
+      <c r="H46" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I46" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="N46" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q46" s="23" t="s">
+        <v>323</v>
+      </c>
+      <c r="R46" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S46" s="28" t="s">
+        <v>324</v>
+      </c>
+      <c r="T46" s="22">
+        <v>1</v>
+      </c>
+      <c r="U46" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V46" s="17">
+        <v>1</v>
+      </c>
+      <c r="W46" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A47" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C47" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E47">
+        <v>38.32</v>
+      </c>
+      <c r="H47" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I47" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="N47" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q47" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R47" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S47" s="28">
+        <v>73108</v>
+      </c>
+      <c r="T47" s="22">
+        <v>1</v>
+      </c>
+      <c r="U47" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V47" s="17">
+        <v>1</v>
+      </c>
+      <c r="W47" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A48" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E48">
+        <v>38.32</v>
+      </c>
+      <c r="H48" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I48" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="N48" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q48" s="23" t="s">
+        <v>325</v>
+      </c>
+      <c r="R48" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S48" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="T48" s="22">
+        <v>1</v>
+      </c>
+      <c r="U48" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V48" s="17">
+        <v>1</v>
+      </c>
+      <c r="W48" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A49" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E49">
+        <v>38.32</v>
+      </c>
+      <c r="H49" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I49" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="N49" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q49" s="23" t="s">
+        <v>327</v>
+      </c>
+      <c r="R49" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S49" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="T49" s="22">
+        <v>1</v>
+      </c>
+      <c r="U49" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V49" s="17">
+        <v>1</v>
+      </c>
+      <c r="W49" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A50" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E50">
+        <v>38.32</v>
+      </c>
+      <c r="H50" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I50" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="N50" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q50" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="R50" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S50" s="28" t="s">
+        <v>330</v>
+      </c>
+      <c r="T50" s="22">
+        <v>1</v>
+      </c>
+      <c r="U50" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V50" s="17">
+        <v>1</v>
+      </c>
+      <c r="W50" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A51" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B51" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51">
+        <v>38.32</v>
+      </c>
+      <c r="H51" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="I51" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="N51" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q51" s="23" t="s">
+        <v>331</v>
+      </c>
+      <c r="R51" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S51" s="28" t="s">
+        <v>332</v>
+      </c>
+      <c r="T51" s="22">
+        <v>1</v>
+      </c>
+      <c r="U51" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V51" s="17">
+        <v>1</v>
+      </c>
+      <c r="W51" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A52" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B52" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52">
+        <v>38.32</v>
+      </c>
+      <c r="H52" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I52" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="N52" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q52" s="23" t="s">
+        <v>333</v>
+      </c>
+      <c r="R52" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S52" s="28" t="s">
+        <v>334</v>
+      </c>
+      <c r="T52" s="22">
+        <v>1</v>
+      </c>
+      <c r="U52" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V52" s="17">
+        <v>1</v>
+      </c>
+      <c r="W52" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A53" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C53" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53">
+        <v>38.32</v>
+      </c>
+      <c r="H53" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I53" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="N53" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="Q53" s="23" t="s">
+        <v>301</v>
+      </c>
+      <c r="R53" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="S53" s="28" t="s">
+        <v>335</v>
+      </c>
+      <c r="T53" s="22">
+        <v>1</v>
+      </c>
+      <c r="U53" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V53" s="17">
+        <v>1</v>
+      </c>
+      <c r="W53" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A54" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C54" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54">
+        <v>38.32</v>
+      </c>
+      <c r="H54" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I54" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="N54" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q54" s="23" t="s">
+        <v>290</v>
+      </c>
+      <c r="R54" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S54" s="28">
+        <v>73069</v>
+      </c>
+      <c r="T54" s="22">
+        <v>1</v>
+      </c>
+      <c r="U54" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V54" s="17">
+        <v>1</v>
+      </c>
+      <c r="W54" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A55" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E55">
+        <v>38.32</v>
+      </c>
+      <c r="H55" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I55" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="N55" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q55" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="R55" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S55" s="28" t="s">
+        <v>336</v>
+      </c>
+      <c r="T55" s="22">
+        <v>1</v>
+      </c>
+      <c r="U55" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V55" s="17">
+        <v>1</v>
+      </c>
+      <c r="W55" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A56" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C56" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E56">
+        <v>38.32</v>
+      </c>
+      <c r="H56" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I56" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="N56" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q56" s="23" t="s">
+        <v>337</v>
+      </c>
+      <c r="R56" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S56" s="28" t="s">
+        <v>338</v>
+      </c>
+      <c r="T56" s="22">
+        <v>1</v>
+      </c>
+      <c r="U56" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V56" s="17">
+        <v>1</v>
+      </c>
+      <c r="W56" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A57" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57">
+        <v>38.32</v>
+      </c>
+      <c r="H57" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I57" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="N57" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q57" s="23" t="s">
+        <v>339</v>
+      </c>
+      <c r="R57" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S57" s="28">
+        <v>49009</v>
+      </c>
+      <c r="T57" s="22">
+        <v>1</v>
+      </c>
+      <c r="U57" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V57" s="17">
+        <v>1</v>
+      </c>
+      <c r="W57" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A58" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B58" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E58">
+        <v>38.32</v>
+      </c>
+      <c r="H58" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I58" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="N58" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q58" s="23" t="s">
+        <v>340</v>
+      </c>
+      <c r="R58" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S58" s="28" t="s">
+        <v>341</v>
+      </c>
+      <c r="T58" s="22">
+        <v>1</v>
+      </c>
+      <c r="U58" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V58" s="17">
+        <v>1</v>
+      </c>
+      <c r="W58" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A59" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B59" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E59">
+        <v>38.32</v>
+      </c>
+      <c r="H59" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I59" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="N59" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q59" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="R59" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S59" s="29" t="s">
+        <v>343</v>
+      </c>
+      <c r="T59" s="22">
+        <v>1</v>
+      </c>
+      <c r="U59" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V59" s="17">
+        <v>1</v>
+      </c>
+      <c r="W59" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A60" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B60" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C60" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E60">
+        <v>38.32</v>
+      </c>
+      <c r="H60" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I60" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="N60" s="23" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q60" s="23" t="s">
+        <v>344</v>
+      </c>
+      <c r="R60" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S60" s="28" t="s">
+        <v>345</v>
+      </c>
+      <c r="T60" s="22">
+        <v>1</v>
+      </c>
+      <c r="U60" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V60" s="17">
+        <v>1</v>
+      </c>
+      <c r="W60" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A61" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B61" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E61">
+        <v>38.32</v>
+      </c>
+      <c r="H61" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I61" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="N61" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q61" s="23" t="s">
+        <v>346</v>
+      </c>
+      <c r="R61" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S61" s="28" t="s">
+        <v>347</v>
+      </c>
+      <c r="T61" s="22">
+        <v>1</v>
+      </c>
+      <c r="U61" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V61" s="17">
+        <v>1</v>
+      </c>
+      <c r="W61" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A62" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B62" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E62">
+        <v>38.32</v>
+      </c>
+      <c r="H62" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I62" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="N62" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q62" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R62" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S62" s="28">
+        <v>73132</v>
+      </c>
+      <c r="T62" s="22">
+        <v>1</v>
+      </c>
+      <c r="U62" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V62" s="17">
+        <v>1</v>
+      </c>
+      <c r="W62" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A63" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B63" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E63">
+        <v>38.32</v>
+      </c>
+      <c r="H63" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I63" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="N63" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q63" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R63" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S63" s="28">
+        <v>73128</v>
+      </c>
+      <c r="T63" s="22">
+        <v>1</v>
+      </c>
+      <c r="U63" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V63" s="17">
+        <v>1</v>
+      </c>
+      <c r="W63" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A64" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B64" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C64" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E64">
+        <v>38.32</v>
+      </c>
+      <c r="H64" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I64" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="N64" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q64" s="25" t="s">
+        <v>348</v>
+      </c>
+      <c r="R64" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S64" s="29">
+        <v>93728</v>
+      </c>
+      <c r="T64" s="22">
+        <v>1</v>
+      </c>
+      <c r="U64" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V64" s="17">
+        <v>1</v>
+      </c>
+      <c r="W64" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A65" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B65" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C65" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E65">
+        <v>38.32</v>
+      </c>
+      <c r="H65" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I65" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="N65" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q65" s="23" t="s">
+        <v>349</v>
+      </c>
+      <c r="R65" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S65" s="28" t="s">
+        <v>350</v>
+      </c>
+      <c r="T65" s="22">
+        <v>1</v>
+      </c>
+      <c r="U65" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V65" s="17">
+        <v>1</v>
+      </c>
+      <c r="W65" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A66" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B66" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E66">
+        <v>38.32</v>
+      </c>
+      <c r="H66" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I66" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="N66" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="Q66" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R66" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S66" s="28">
+        <v>73112</v>
+      </c>
+      <c r="T66" s="22">
+        <v>1</v>
+      </c>
+      <c r="U66" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V66" s="17">
+        <v>1</v>
+      </c>
+      <c r="W66" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A67" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B67" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="H67" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="I67" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="N67" s="24" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q67" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="R67" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="S67" s="31" t="s">
+        <v>351</v>
+      </c>
+      <c r="T67" s="22">
+        <v>1</v>
+      </c>
+      <c r="U67" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V67" s="17">
+        <v>1</v>
+      </c>
+      <c r="W67" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A68" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B68" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E68">
+        <v>38.32</v>
+      </c>
+      <c r="H68" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="I68" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="N68" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q68" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="R68" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S68" s="28">
+        <v>21215</v>
+      </c>
+      <c r="T68" s="22">
+        <v>1</v>
+      </c>
+      <c r="U68" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V68" s="17">
+        <v>1</v>
+      </c>
+      <c r="W68" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A69" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E69">
+        <v>38.32</v>
+      </c>
+      <c r="H69" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I69" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="N69" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q69" s="23" t="s">
+        <v>352</v>
+      </c>
+      <c r="R69" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S69" s="28">
+        <v>78148</v>
+      </c>
+      <c r="T69" s="22">
+        <v>1</v>
+      </c>
+      <c r="U69" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V69" s="17">
+        <v>1</v>
+      </c>
+      <c r="W69" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A70" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B70" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E70">
+        <v>38.32</v>
+      </c>
+      <c r="H70" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I70" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="N70" s="23" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q70" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R70" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S70" s="28">
+        <v>73134</v>
+      </c>
+      <c r="T70" s="22">
+        <v>1</v>
+      </c>
+      <c r="U70" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V70" s="17">
+        <v>1</v>
+      </c>
+      <c r="W70" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A71" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B71" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E71">
+        <v>38.32</v>
+      </c>
+      <c r="H71" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="I71" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="N71" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q71" s="23" t="s">
+        <v>353</v>
+      </c>
+      <c r="R71" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="S71" s="28">
+        <v>61832</v>
+      </c>
+      <c r="T71" s="22">
+        <v>1</v>
+      </c>
+      <c r="U71" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V71" s="17">
+        <v>1</v>
+      </c>
+      <c r="W71" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A72" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B72" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C72" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E72">
+        <v>38.32</v>
+      </c>
+      <c r="H72" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I72" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="N72" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q72" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="R72" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S72" s="29" t="s">
+        <v>355</v>
+      </c>
+      <c r="T72" s="22">
+        <v>1</v>
+      </c>
+      <c r="U72" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V72" s="17">
+        <v>1</v>
+      </c>
+      <c r="W72" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A73" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C73" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E73">
+        <v>38.32</v>
+      </c>
+      <c r="H73" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I73" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="N73" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q73" s="23" t="s">
+        <v>356</v>
+      </c>
+      <c r="R73" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S73" s="28">
+        <v>95403</v>
+      </c>
+      <c r="T73" s="22">
+        <v>1</v>
+      </c>
+      <c r="U73" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V73" s="17">
+        <v>1</v>
+      </c>
+      <c r="W73" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A74" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B74" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C74" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E74">
+        <v>38.32</v>
+      </c>
+      <c r="H74" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I74" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="N74" s="23" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q74" s="23" t="s">
+        <v>357</v>
+      </c>
+      <c r="R74" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S74" s="28">
+        <v>73099</v>
+      </c>
+      <c r="T74" s="22">
+        <v>1</v>
+      </c>
+      <c r="U74" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V74" s="17">
+        <v>1</v>
+      </c>
+      <c r="W74" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A75" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B75" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C75" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E75">
+        <v>38.32</v>
+      </c>
+      <c r="H75" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I75" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="N75" s="23" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q75" s="23" t="s">
+        <v>358</v>
+      </c>
+      <c r="R75" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S75" s="28">
+        <v>49202</v>
+      </c>
+      <c r="T75" s="22">
+        <v>1</v>
+      </c>
+      <c r="U75" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V75" s="17">
+        <v>1</v>
+      </c>
+      <c r="W75" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A76" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B76" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C76" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E76">
+        <v>38.32</v>
+      </c>
+      <c r="H76" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I76" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="N76" s="23" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q76" s="23" t="s">
+        <v>359</v>
+      </c>
+      <c r="R76" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S76" s="28" t="s">
+        <v>360</v>
+      </c>
+      <c r="T76" s="22">
+        <v>1</v>
+      </c>
+      <c r="U76" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V76" s="17">
+        <v>1</v>
+      </c>
+      <c r="W76" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A77" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B77" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E77">
+        <v>38.32</v>
+      </c>
+      <c r="H77" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I77" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="N77" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q77" s="23" t="s">
+        <v>361</v>
+      </c>
+      <c r="R77" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S77" s="28" t="s">
+        <v>362</v>
+      </c>
+      <c r="T77" s="22">
+        <v>1</v>
+      </c>
+      <c r="U77" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V77" s="17">
+        <v>1</v>
+      </c>
+      <c r="W77" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A78" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E78">
+        <v>38.32</v>
+      </c>
+      <c r="H78" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I78" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="N78" s="23" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q78" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R78" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S78" s="28">
+        <v>73127</v>
+      </c>
+      <c r="T78" s="22">
+        <v>1</v>
+      </c>
+      <c r="U78" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V78" s="17">
+        <v>1</v>
+      </c>
+      <c r="W78" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A79" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B79" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C79" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E79">
+        <v>38.32</v>
+      </c>
+      <c r="H79" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I79" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="N79" s="23" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q79" s="23" t="s">
+        <v>363</v>
+      </c>
+      <c r="R79" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S79" s="28" t="s">
+        <v>364</v>
+      </c>
+      <c r="T79" s="22">
+        <v>1</v>
+      </c>
+      <c r="U79" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V79" s="17">
+        <v>1</v>
+      </c>
+      <c r="W79" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A80" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B80" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C80" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E80">
+        <v>38.32</v>
+      </c>
+      <c r="H80" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I80" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="N80" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q80" s="23" t="s">
+        <v>365</v>
+      </c>
+      <c r="R80" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="S80" s="28" t="s">
+        <v>366</v>
+      </c>
+      <c r="T80" s="22">
+        <v>1</v>
+      </c>
+      <c r="U80" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V80" s="17">
+        <v>1</v>
+      </c>
+      <c r="W80" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A81" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B81" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C81" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E81">
+        <v>38.32</v>
+      </c>
+      <c r="H81" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I81" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="N81" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="Q81" s="23" t="s">
+        <v>325</v>
+      </c>
+      <c r="R81" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="S81" s="28" t="s">
+        <v>367</v>
+      </c>
+      <c r="T81" s="22">
+        <v>1</v>
+      </c>
+      <c r="U81" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V81" s="17">
+        <v>1</v>
+      </c>
+      <c r="W81" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A82" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B82" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C82" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E82">
+        <v>38.32</v>
+      </c>
+      <c r="H82" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="I82" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="N82" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q82" s="25" t="s">
+        <v>368</v>
+      </c>
+      <c r="R82" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S82" s="29" t="s">
+        <v>369</v>
+      </c>
+      <c r="T82" s="22">
+        <v>1</v>
+      </c>
+      <c r="U82" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V82" s="17">
+        <v>1</v>
+      </c>
+      <c r="W82" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A83" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B83" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C83" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E83">
+        <v>38.32</v>
+      </c>
+      <c r="H83" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="I83" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="N83" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q83" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="R83" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="S83" s="29" t="s">
+        <v>371</v>
+      </c>
+      <c r="T83" s="22">
+        <v>1</v>
+      </c>
+      <c r="U83" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V83" s="17">
+        <v>1</v>
+      </c>
+      <c r="W83" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A84" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B84" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E84">
+        <v>38.32</v>
+      </c>
+      <c r="H84" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I84" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="N84" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q84" s="23" t="s">
+        <v>372</v>
+      </c>
+      <c r="R84" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="S84" s="28" t="s">
+        <v>373</v>
+      </c>
+      <c r="T84" s="22">
+        <v>1</v>
+      </c>
+      <c r="U84" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V84" s="17">
+        <v>1</v>
+      </c>
+      <c r="W84" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A85" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B85" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C85" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E85">
+        <v>38.32</v>
+      </c>
+      <c r="H85" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I85" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="N85" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q85" s="23" t="s">
+        <v>374</v>
+      </c>
+      <c r="R85" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S85" s="28">
+        <v>94928</v>
+      </c>
+      <c r="T85" s="22">
+        <v>1</v>
+      </c>
+      <c r="U85" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V85" s="17">
+        <v>1</v>
+      </c>
+      <c r="W85" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A86" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B86" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C86" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E86">
+        <v>38.32</v>
+      </c>
+      <c r="H86" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="I86" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="N86" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q86" s="23" t="s">
+        <v>375</v>
+      </c>
+      <c r="R86" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S86" s="28">
+        <v>76201</v>
+      </c>
+      <c r="T86" s="22">
+        <v>1</v>
+      </c>
+      <c r="U86" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V86" s="17">
+        <v>1</v>
+      </c>
+      <c r="W86" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A87" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B87" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C87" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E87">
+        <v>38.32</v>
+      </c>
+      <c r="H87" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I87" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="N87" s="23" t="s">
+        <v>242</v>
+      </c>
+      <c r="Q87" s="23" t="s">
+        <v>376</v>
+      </c>
+      <c r="R87" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S87" s="28">
+        <v>95367</v>
+      </c>
+      <c r="T87" s="22">
+        <v>1</v>
+      </c>
+      <c r="U87" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V87" s="17">
+        <v>1</v>
+      </c>
+      <c r="W87" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A88" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B88" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C88" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E88">
+        <v>38.32</v>
+      </c>
+      <c r="H88" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I88" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="N88" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="Q88" s="23" t="s">
+        <v>377</v>
+      </c>
+      <c r="R88" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S88" s="28" t="s">
+        <v>378</v>
+      </c>
+      <c r="T88" s="22">
+        <v>1</v>
+      </c>
+      <c r="U88" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V88" s="17">
+        <v>1</v>
+      </c>
+      <c r="W88" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A89" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B89" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C89" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E89">
+        <v>38.32</v>
+      </c>
+      <c r="H89" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I89" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="N89" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q89" s="23" t="s">
+        <v>379</v>
+      </c>
+      <c r="R89" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S89" s="28" t="s">
+        <v>380</v>
+      </c>
+      <c r="T89" s="22">
+        <v>1</v>
+      </c>
+      <c r="U89" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V89" s="17">
+        <v>1</v>
+      </c>
+      <c r="W89" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A90" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B90" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C90" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E90">
+        <v>38.32</v>
+      </c>
+      <c r="H90" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I90" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="N90" s="23" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q90" s="23" t="s">
+        <v>381</v>
+      </c>
+      <c r="R90" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S90" s="28" t="s">
+        <v>382</v>
+      </c>
+      <c r="T90" s="22">
+        <v>1</v>
+      </c>
+      <c r="U90" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V90" s="17">
+        <v>1</v>
+      </c>
+      <c r="W90" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A91" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B91" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C91" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E91">
+        <v>38.32</v>
+      </c>
+      <c r="H91" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I91" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="N91" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q91" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R91" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S91" s="28">
+        <v>73115</v>
+      </c>
+      <c r="T91" s="22">
+        <v>1</v>
+      </c>
+      <c r="U91" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V91" s="17">
+        <v>1</v>
+      </c>
+      <c r="W91" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A92" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B92" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C92" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E92">
+        <v>38.32</v>
+      </c>
+      <c r="H92" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I92" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="N92" s="23" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q92" s="23" t="s">
+        <v>357</v>
+      </c>
+      <c r="R92" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S92" s="28">
+        <v>73099</v>
+      </c>
+      <c r="T92" s="22">
+        <v>1</v>
+      </c>
+      <c r="U92" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V92" s="17">
+        <v>1</v>
+      </c>
+      <c r="W92" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A93" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B93" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C93" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E93">
+        <v>38.32</v>
+      </c>
+      <c r="H93" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="I93" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="N93" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="Q93" s="23" t="s">
+        <v>383</v>
+      </c>
+      <c r="R93" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S93" s="28">
+        <v>20783</v>
+      </c>
+      <c r="T93" s="22">
+        <v>1</v>
+      </c>
+      <c r="U93" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V93" s="17">
+        <v>1</v>
+      </c>
+      <c r="W93" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A94" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B94" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C94" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E94">
+        <v>38.32</v>
+      </c>
+      <c r="H94" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I94" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="N94" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q94" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="R94" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="S94" s="28" t="s">
+        <v>385</v>
+      </c>
+      <c r="T94" s="22">
+        <v>1</v>
+      </c>
+      <c r="U94" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V94" s="17">
+        <v>1</v>
+      </c>
+      <c r="W94" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A95" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B95" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C95" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E95">
+        <v>38.32</v>
+      </c>
+      <c r="H95" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I95" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="N95" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q95" s="25" t="s">
+        <v>386</v>
+      </c>
+      <c r="R95" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S95" s="29" t="s">
+        <v>387</v>
+      </c>
+      <c r="T95" s="22">
+        <v>1</v>
+      </c>
+      <c r="U95" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V95" s="17">
+        <v>1</v>
+      </c>
+      <c r="W95" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A96" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B96" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C96" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E96">
+        <v>38.32</v>
+      </c>
+      <c r="H96" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I96" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="N96" s="23" t="s">
+        <v>251</v>
+      </c>
+      <c r="Q96" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R96" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S96" s="28">
+        <v>73110</v>
+      </c>
+      <c r="T96" s="22">
+        <v>1</v>
+      </c>
+      <c r="U96" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V96" s="17">
+        <v>1</v>
+      </c>
+      <c r="W96" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A97" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B97" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C97" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E97">
+        <v>38.32</v>
+      </c>
+      <c r="H97" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I97" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="N97" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q97" s="23" t="s">
+        <v>388</v>
+      </c>
+      <c r="R97" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="S97" s="28" t="s">
+        <v>389</v>
+      </c>
+      <c r="T97" s="22">
+        <v>1</v>
+      </c>
+      <c r="U97" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V97" s="17">
+        <v>1</v>
+      </c>
+      <c r="W97" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A98" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B98" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C98" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E98">
+        <v>38.32</v>
+      </c>
+      <c r="H98" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="I98" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="N98" s="25" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q98" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="R98" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S98" s="29">
+        <v>95148</v>
+      </c>
+      <c r="T98" s="22">
+        <v>1</v>
+      </c>
+      <c r="U98" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V98" s="17">
+        <v>1</v>
+      </c>
+      <c r="W98" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A99" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B99" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C99" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E99">
+        <v>38.32</v>
+      </c>
+      <c r="H99" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I99" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="N99" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="Q99" s="23" t="s">
+        <v>390</v>
+      </c>
+      <c r="R99" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S99" s="28" t="s">
+        <v>391</v>
+      </c>
+      <c r="T99" s="22">
+        <v>1</v>
+      </c>
+      <c r="U99" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V99" s="17">
+        <v>1</v>
+      </c>
+      <c r="W99" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A100" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B100" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C100" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E100">
+        <v>38.32</v>
+      </c>
+      <c r="H100" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I100" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="N100" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="Q100" s="23" t="s">
+        <v>392</v>
+      </c>
+      <c r="R100" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="S100" s="28" t="s">
+        <v>393</v>
+      </c>
+      <c r="T100" s="22">
+        <v>1</v>
+      </c>
+      <c r="U100" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V100" s="17">
+        <v>1</v>
+      </c>
+      <c r="W100" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A101" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B101" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C101" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E101">
+        <v>38.32</v>
+      </c>
+      <c r="H101" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="I101" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="N101" s="23" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q101" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="R101" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="S101" s="28">
+        <v>73112</v>
+      </c>
+      <c r="T101" s="22">
+        <v>1</v>
+      </c>
+      <c r="U101" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V101" s="17">
+        <v>1</v>
+      </c>
+      <c r="W101" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A102" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B102" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C102" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E102">
+        <v>38.32</v>
+      </c>
+      <c r="H102" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I102" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="N102" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q102" s="25" t="s">
+        <v>394</v>
+      </c>
+      <c r="R102" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="S102" s="29" t="s">
+        <v>395</v>
+      </c>
+      <c r="T102" s="22">
+        <v>1</v>
+      </c>
+      <c r="U102" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V102" s="17">
+        <v>1</v>
+      </c>
+      <c r="W102" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A103" s="14">
+        <v>45973</v>
+      </c>
+      <c r="B103" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C103" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E103">
+        <v>38.32</v>
+      </c>
+      <c r="H103" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I103" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="N103" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="Q103" s="23" t="s">
+        <v>396</v>
+      </c>
+      <c r="R103" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S103" s="28" t="s">
+        <v>397</v>
+      </c>
+      <c r="T103" s="22">
+        <v>1</v>
+      </c>
+      <c r="U103" s="17">
+        <v>108692</v>
+      </c>
+      <c r="V103" s="17">
+        <v>1</v>
+      </c>
+      <c r="W103" s="17">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:W3">
-    <sortCondition ref="I2:I3"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S3">
+    <sortCondition ref="F2:F3"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>